<commit_message>
Seleniumbase code sample added
</commit_message>
<xml_diff>
--- a/data/TestData.xlsx
+++ b/data/TestData.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -539,17 +539,17 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>chromium</t>
+          <t>chrome</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>chromium</t>
+          <t>chrome</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>chromium</t>
+          <t>chrome</t>
         </is>
       </c>
     </row>
@@ -770,6 +770,28 @@
       <c r="D13" s="3" t="inlineStr">
         <is>
           <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GOOGLE_URL</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://google.com</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://google.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://google.com</t>
         </is>
       </c>
     </row>

</xml_diff>